<commit_message>
Atualiza exemplo de vencimentos pra 3 bankers
config/vencimentos.example.xlsx ganhou 3 vencimentos a mais pro
banker fictício "Ciclano Nunes", espalhados em meses diferentes
(set/out/dez), pra manter a mesma quantidade de bankers de exemplo
usada em config/saldos.example.xlsx (Fulano Silva, Beltrano Souza,
Ciclano Nunes).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QWgeXNNmjYVnh184fZ5Ac9
</commit_message>
<xml_diff>
--- a/config/vencimentos.example.xlsx
+++ b/config/vencimentos.example.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -416,8 +416,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -457,10 +466,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>001111111</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1111111</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -488,10 +495,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>002222222</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2222222</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -519,10 +524,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>003333333</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3333333</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -550,10 +553,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>004444444</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4444444</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -581,10 +582,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>005555555</t>
-        </is>
+      <c r="A6" t="n">
+        <v>5555555</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -608,6 +607,93 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>Beltrano Souza</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6666666</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>STU_VW</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CDB</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>8200</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Ciclano Nunes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7777777</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>XYZ_AB</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>LCA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4150.5</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Ciclano Nunes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8888888</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CDE_FG</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TESOURO DIRETO - SELIC</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>21000</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>46368</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Ciclano Nunes</t>
         </is>
       </c>
     </row>

</xml_diff>